<commit_message>
Include Gherkin PT-BR in Description field of Azure import files
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015uoCdPRJWqErwK3dazSzro
</commit_message>
<xml_diff>
--- a/docs/azure-import/test-cases-1276695.xlsx
+++ b/docs/azure-import/test-cases-1276695.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -438,6 +438,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,6 +482,11 @@
           <t>Tags</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr"/>
@@ -513,6 +519,11 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Parametrização de travas de parecer na T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Configurar tempo mínimo e quantidade máxima por especialidade detalhe e filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador com acesso à T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando configuro tempo mínimo em horas e quantidade máxima para uma especialidade detalhe em uma filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E salvo a parametrização&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então os valores ficam armazenados vinculados à combinação especialidade detalhe x filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a alteração é registrada no histórico com usuário, data/hora e valores anterior e atual</t>
         </is>
       </c>
     </row>
@@ -535,6 +546,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr"/>
@@ -555,6 +567,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr"/>
@@ -587,6 +600,11 @@
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Configurar faixa etária por especialidade detalhe e filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador com acesso à T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando defino idade mínima e idade máxima para uma especialidade detalhe em uma filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema armazena a faixa etária vinculada à combinação especialidade detalhe x filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a alteração é registrada no histórico</t>
         </is>
       </c>
     </row>
@@ -609,6 +627,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr"/>
@@ -641,6 +660,11 @@
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D4</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Configurar limite de frequência com comportamento ao atingir&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador com acesso à T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando configuro quantidade máxima &amp;lt;qtd&amp;gt;, intervalo de &amp;lt;horas&amp;gt; horas e comportamento "&amp;lt;comportamento&amp;gt;"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema aceita e armazena os valores&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E registra a alteração no histórico com usuário, data/hora e valores anterior e atual&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| qtd | horas | comportamento                      |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3   | 24    | Com justificativa                  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 2   | 48    | Sem justificativa (Trava Total)    |</t>
         </is>
       </c>
     </row>
@@ -663,6 +687,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr"/>
@@ -683,6 +708,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr"/>
@@ -703,6 +729,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
@@ -735,6 +762,11 @@
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Registrar histórico de todas as alterações da parametrização&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que uma especialidade detalhe possui tempo mínimo 24 configurado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando altero o tempo mínimo para 48 e a faixa etária máxima&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o histórico exibe um registro por campo alterado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E cada registro contém usuário, data/hora, valor anterior e valor atual</t>
         </is>
       </c>
     </row>
@@ -757,6 +789,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr"/>
@@ -789,6 +822,11 @@
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D14</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Assumir 0 quando a quantidade não é informada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador na T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando salvo uma especialidade detalhe sem informar a quantidade máxima&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o campo é gravado com o valor 0</t>
         </is>
       </c>
     </row>
@@ -811,6 +849,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr"/>
@@ -843,6 +882,11 @@
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Permitir solicitação sem parametrização de tempo ou limite&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade detalhe x filial não possui tempo mínimo nem limite de frequência&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita teleparecer dessa especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema permite a solicitação normalmente, sem restrição</t>
         </is>
       </c>
     </row>
@@ -865,6 +909,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr"/>
@@ -897,6 +942,11 @@
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D1</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Usar o Controle de Tempo geral quando a especialidade não tem tempo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade detalhe não possui tempo parametrizado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o Controle de Tempo geral é de 48 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que existe solicitação da especialidade há 10 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar novamente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema considera o tempo de 48 horas do Controle de Tempo geral</t>
         </is>
       </c>
     </row>
@@ -919,6 +969,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr"/>
@@ -951,6 +1002,11 @@
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Contar o tempo a partir da data/hora da solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o tempo mínimo é de 24 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que existe parecer solicitado às 08:00 com status &amp;lt;status&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que foi respondido/cancelado às 20:00&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico consulta a opção às 10:00 do mesmo dia&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o tempo restante exibido é "22h 0min" contado a partir das 08:00&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| status    |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| Finalizado |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| Pendente  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| Cancelado |</t>
         </is>
       </c>
     </row>
@@ -973,6 +1029,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr"/>
@@ -993,6 +1050,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr"/>
@@ -1013,6 +1071,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr"/>
@@ -1033,6 +1092,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr"/>
@@ -1065,6 +1125,11 @@
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Manter a trava de solicitação em andamento no mesmo atendimento&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe solicitação em andamento/pendente da especialidade no mesmo atendimento&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar novamente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então prevalece o comportamento atual do sistema (solicitação não permitida)</t>
         </is>
       </c>
     </row>
@@ -1087,6 +1152,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr"/>
@@ -1119,6 +1185,11 @@
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D14</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Aplicar parametrização diferente por filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a filial A tem tempo mínimo de 24 horas e a filial B tem 6 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que existe parecer da especialidade há 10 horas no paciente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico da filial A e o médico da filial B consultam a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então na filial A a opção está bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E na filial B a opção está habilitada</t>
         </is>
       </c>
     </row>
@@ -1141,6 +1212,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr"/>
@@ -1173,6 +1245,11 @@
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D14</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Rejeitar valores inválidos&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador na T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando informo &amp;lt;campo&amp;gt; = "&amp;lt;valor&amp;gt;"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema &amp;lt;resultado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| campo             | valor | resultado                     |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| tempo mínimo      | -1    | rejeita o valor               |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| quantidade máxima | abc   | rejeita o valor               |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| idade mínima maior que a máxima | 60 / 18 | rejeita o valor |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| tempo mínimo      | 0     | conforme definição do PO      |</t>
         </is>
       </c>
     </row>
@@ -1195,6 +1272,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr"/>
@@ -1215,6 +1293,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr"/>
@@ -1235,6 +1314,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr"/>
@@ -1255,6 +1335,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr"/>
@@ -1275,6 +1356,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr"/>
@@ -1307,6 +1389,11 @@
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Configurar janela de horas do lembrete de parecer recente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que sou um administrador na T41TRAVA&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando informo a janela de horas do lembrete para uma especialidade detalhe x filial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o valor é gravado de forma independente do limite de frequência&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a alteração é registrada no histórico</t>
         </is>
       </c>
     </row>
@@ -1329,6 +1416,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr"/>
@@ -1361,6 +1449,11 @@
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Validação de multiplicidade e faixa etária na solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Permitir solicitação sem restrições&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que não existe parecer recente da especialidade dentro do intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que a idade do paciente está dentro da faixa etária configurada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a opção de teleparecer/parecer presencial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema permite a solicitação normalmente</t>
         </is>
       </c>
     </row>
@@ -1383,6 +1476,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr"/>
@@ -1403,6 +1497,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr"/>
@@ -1435,6 +1530,11 @@
       <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D5</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Bloquear por parecer recente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe parecer da mesma especialidade detalhe dentro do intervalo configurado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a opção de teleparecer/parecer presencial&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então é exibida modal "ATENÇÃO! ESSE PARECER JÁ FOI SOLICITADO."&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o texto informa a data da solicitação anterior&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E informa "Será possível solicitar um novo parecer em: Xh Ymin"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E lista os pareceres da mesma especialidade com formato, especialidade, solicitado em, solicitante, status e botão "Abrir parecer"</t>
         </is>
       </c>
     </row>
@@ -1457,6 +1557,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr"/>
@@ -1477,6 +1578,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr"/>
@@ -1509,6 +1611,11 @@
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D5; D6</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Exibir tooltip com motivo e tempo restante&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a opção está bloqueada por parecer recente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico passa o mouse sobre a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o tooltip exibe o motivo do bloqueio&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E exibe o tempo restante no formato "Xh Ymin"</t>
         </is>
       </c>
     </row>
@@ -1531,6 +1638,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr"/>
@@ -1563,6 +1671,11 @@
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Validar a virada do intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o intervalo configurado é de 24 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o parecer anterior foi solicitado há &amp;lt;tempo&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a Solicitação de Pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção está &amp;lt;estado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o tempo restante exibido é &amp;lt;restante&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| tempo     | estado       | restante |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 23h 59min | bloqueada    | 0h 1min  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 24h 00min | habilitada   | -        |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 24h 01min | habilitada   | -        |</t>
         </is>
       </c>
     </row>
@@ -1585,6 +1698,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr"/>
@@ -1605,6 +1719,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr"/>
@@ -1625,6 +1740,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr"/>
@@ -1645,6 +1761,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr"/>
@@ -1677,6 +1794,11 @@
       <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D2</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Desabilitar opção fora da faixa etária&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a idade do paciente está fora da faixa etária da especialidade detalhe&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico visualiza a lista de opções&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção aparece desabilitada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E ao passar o mouse aparece "Especialidade não disponível para a faixa etária do paciente"</t>
         </is>
       </c>
     </row>
@@ -1699,6 +1821,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr"/>
@@ -1731,6 +1854,11 @@
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D7</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Validar limites de idade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a faixa etária é de &amp;lt;mín&amp;gt; a &amp;lt;máx&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o paciente possui &amp;lt;idade&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a Solicitação de Pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção está &amp;lt;estado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| mín     | máx     | idade             | estado       |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 18 anos | 59 anos | 17 anos 11 meses  | desabilitada |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 18 anos | 59 anos | 18 anos           | habilitada   |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 18 anos | 59 anos | 59 anos           | habilitada   |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 18 anos | 59 anos | 60 anos           | desabilitada |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 0 meses | 12 meses| 13 meses          | desabilitada |</t>
         </is>
       </c>
     </row>
@@ -1753,6 +1881,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr"/>
@@ -1773,6 +1902,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr"/>
@@ -1793,6 +1923,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr"/>
@@ -1813,6 +1944,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr"/>
@@ -1833,6 +1965,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr"/>
@@ -1853,6 +1986,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr"/>
@@ -1885,6 +2019,11 @@
       <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Exibir opção sem regra de faixa etária&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade detalhe x filial não possui faixa etária configurada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o paciente possui &amp;lt;idade&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico visualiza a lista&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção está habilitada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| idade   |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 2 dias  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 10 anos |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 90 anos |</t>
         </is>
       </c>
     </row>
@@ -1907,6 +2046,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr"/>
@@ -1927,6 +2067,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr"/>
@@ -1947,6 +2088,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr"/>
@@ -1967,6 +2109,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr"/>
@@ -1999,6 +2142,11 @@
       <c r="H63" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D1</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Não aplicar restrição temporal sem tempo mínimo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade detalhe x filial não possui tempo mínimo configurado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que existe parecer recente da especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a solicitação é permitida normalmente</t>
         </is>
       </c>
     </row>
@@ -2021,6 +2169,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr"/>
@@ -2053,6 +2202,11 @@
       <c r="H65" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D3</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Exibir modal ao atingir o limite com comportamento "Com justificativa"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite de solicitações foi atingido no intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o comportamento parametrizado é "Com justificativa"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta selecionar a opção bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema exibe modal informando o limite atingido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o modal apresenta os campos de justificativa e de caso clínico obrigatório&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E apresenta a quantidade já solicitada e o saldo restante</t>
         </is>
       </c>
     </row>
@@ -2075,6 +2229,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr"/>
@@ -2107,6 +2262,11 @@
       <c r="H67" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Impedir a solicitação em Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite de solicitações foi atingido no intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o comportamento parametrizado é "Sem justificativa (Trava Total)"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta selecionar a opção bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema impede completamente a solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E oferece a visualização dos pareceres anteriores respondidos&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E não permite prosseguir enquanto o intervalo não for cumprido</t>
         </is>
       </c>
     </row>
@@ -2129,6 +2289,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr"/>
@@ -2161,6 +2322,11 @@
       <c r="H69" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D10</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Exibir e atualizar o saldo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite é &amp;lt;limite&amp;gt; em &amp;lt;horas&amp;gt; horas e já foram solicitados &amp;lt;usados&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a Solicitação de Pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então é exibido "Você ainda pode solicitar &amp;lt;saldo&amp;gt; parecer(es) nas próximas &amp;lt;horas&amp;gt;h"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| limite | horas | usados | saldo |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 24    | 0      | 3     |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 24    | 1      | 2     |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 24    | 3      | 0     |</t>
         </is>
       </c>
     </row>
@@ -2183,6 +2349,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr"/>
@@ -2203,6 +2370,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr"/>
       <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr"/>
@@ -2223,6 +2391,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr"/>
@@ -2243,6 +2412,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr"/>
@@ -2275,6 +2445,11 @@
       <c r="H74" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D4</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Tratar parecer não respondido como pendente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe parecer solicitado e ainda não respondido dentro do intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar novo parecer da mesma especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema aplica a Trava Total e bloqueia completamente a solicitação</t>
         </is>
       </c>
     </row>
@@ -2297,6 +2472,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr"/>
@@ -2329,6 +2505,11 @@
       <c r="H76" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Considerar parecer cancelado na verificação da trava&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe parecer da especialidade cancelado dentro do intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema aplica o bloqueio da regra já existente para parecer cancelado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E essa verificação ocorre antes das novas regras</t>
         </is>
       </c>
     </row>
@@ -2351,6 +2532,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr"/>
@@ -2383,6 +2565,11 @@
       <c r="H78" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Priorizar as travas existentes sobre as novas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe solicitação em andamento no mesmo atendimento&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que a especialidade também está bloqueada pelo limite de frequência&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então prevalece o comportamento atual da trava existente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a mensagem das novas regras não é exibida</t>
         </is>
       </c>
     </row>
@@ -2405,6 +2592,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr"/>
@@ -2437,6 +2625,11 @@
       <c r="H80" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Contar pareceres de outros atendimentos do mesmo paciente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o paciente teve pareceres da especialidade em outro atendimento dentro do intervalo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita no atendimento atual&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a contagem considera os pareceres do prontuário do paciente</t>
         </is>
       </c>
     </row>
@@ -2459,6 +2652,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr"/>
@@ -2491,6 +2685,11 @@
       <c r="H82" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D8</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Exibir motivo com mais de um bloqueio&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a opção está bloqueada por parecer recente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que a idade do paciente está fora da faixa etária&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico passa o mouse sobre a opção&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o tooltip exibe o motivo conforme a precedência definida pelo PO</t>
         </is>
       </c>
     </row>
@@ -2513,6 +2712,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr"/>
@@ -2545,6 +2745,11 @@
       <c r="H84" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D11</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Registrar tentativa de solicitação bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o médico tentou solicitar uma opção bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando consulto o log de auditoria&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então há registro da tentativa com usuário, paciente, especialidade detalhe e data/hora</t>
         </is>
       </c>
     </row>
@@ -2567,6 +2772,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr"/>
@@ -2599,6 +2805,11 @@
       <c r="H86" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D3</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Modal de justificativa e caso clínico&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Exibir a modal com limite, campos e saldo&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite foi atingido e o comportamento é "Com justificativa"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta prosseguir com a solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a modal informa que o limite foi atingido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E exibe a quantidade já utilizada e o saldo restante&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E exibe o campo de justificativa e o campo de caso clínico</t>
         </is>
       </c>
     </row>
@@ -2621,6 +2832,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr"/>
@@ -2653,6 +2865,11 @@
       <c r="H88" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Exibir somente justificativas ativas com "Outro" ao final&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existem justificativas Ativas e Inativas cadastradas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a lista de justificativas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então somente as Ativas são exibidas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a opção "Outro" aparece sempre por último</t>
         </is>
       </c>
     </row>
@@ -2675,6 +2892,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr"/>
@@ -2707,6 +2925,11 @@
       <c r="H90" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Exigir texto livre ao selecionar "Outro"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado a modal de justificativa aberta&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona "Outro"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então é exibido campo de texto livre obrigatório&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E não é possível confirmar sem preenchê-lo</t>
         </is>
       </c>
     </row>
@@ -2729,6 +2952,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr"/>
@@ -2761,6 +2985,11 @@
       <c r="H92" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D3</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Confirmar somente com os dois campos&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado a modal de justificativa aberta&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico preenche justificativa "&amp;lt;just&amp;gt;" e caso clínico "&amp;lt;caso&amp;gt;"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a confirmação da solicitação é &amp;lt;resultado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| just          | caso          | resultado  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| vazia         | vazio         | bloqueada  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| preenchida    | vazio         | bloqueada  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| vazia         | preenchido    | bloqueada  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| só espaços    | preenchido    | bloqueada  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| preenchida    | preenchido    | permitida  |</t>
         </is>
       </c>
     </row>
@@ -2783,6 +3012,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr"/>
@@ -2803,6 +3033,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr"/>
@@ -2823,6 +3054,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr"/>
@@ -2843,6 +3075,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr"/>
@@ -2863,6 +3096,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr"/>
@@ -2883,6 +3117,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr"/>
@@ -2915,6 +3150,11 @@
       <c r="H99" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Registrar justificativa e caso clínico&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o médico confirmou a solicitação com justificativa e caso clínico&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando consulto o log de auditoria&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então há registro com justificativa, caso clínico, usuário, data/hora e especialidade detalhe</t>
         </is>
       </c>
     </row>
@@ -2937,6 +3177,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr"/>
@@ -2969,6 +3210,11 @@
       <c r="H101" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D14</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Inativar sim, excluir não&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe uma justificativa cadastrada &amp;lt;tipo&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o administrador tenta &amp;lt;ação&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema &amp;lt;resultado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| tipo       | ação      | resultado          |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| comum      | inativar  | permite            |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| comum      | excluir   | não permite        |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| "Outro"    | inativar  | não permite        |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| "Outro"    | remover   | não permite        |</t>
         </is>
       </c>
     </row>
@@ -2991,6 +3237,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr"/>
@@ -3011,6 +3258,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr"/>
@@ -3031,6 +3279,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr"/>
@@ -3051,6 +3300,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr"/>
       <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr"/>
@@ -3071,6 +3321,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr"/>
@@ -3103,6 +3354,11 @@
       <c r="H107" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Não exibir a modal na Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite foi atingido e o comportamento é "Sem justificativa (Trava Total)"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a modal de justificativa não é exibida</t>
         </is>
       </c>
     </row>
@@ -3125,6 +3381,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr"/>
@@ -3157,6 +3414,11 @@
       <c r="H109" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Visualização de pareceres anteriores na Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Consultar pareceres anteriores em modo somente leitura&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a solicitação está em Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico aciona "Abrir parecer"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então são listados os pareceres respondidos da especialidade dentro do período&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E cada parecer exibe data e hora, nome do parecerista, CRM e conteúdo da resposta&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a visualização é somente leitura, sem edição nem exclusão</t>
         </is>
       </c>
     </row>
@@ -3179,6 +3441,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr"/>
@@ -3211,6 +3474,11 @@
       <c r="H111" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D6</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Manter a nova solicitação bloqueada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a solicitação está em Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta iniciar nova solicitação da especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o botão/opção permanece completamente bloqueado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E é exibido o tempo restante no formato "Xh Ymin"</t>
         </is>
       </c>
     </row>
@@ -3233,6 +3501,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr"/>
@@ -3265,6 +3534,11 @@
       <c r="H113" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Informar ausência de pareceres respondidos&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite foi atingido apenas com pareceres pendentes&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta visualizar pareceres anteriores&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então é exibida mensagem informando que não há pareceres anteriores disponíveis&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a trava permanece ativa</t>
         </is>
       </c>
     </row>
@@ -3287,6 +3561,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr"/>
@@ -3319,6 +3594,11 @@
       <c r="H115" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D2</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Bloqueio por faixa etária no Siga Internação&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Desabilitar opção e exibir tooltip&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade detalhe possui faixa etária parametrizada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o paciente está fora dessa faixa&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico acessa "Exames, procedimentos e pareceres" &amp;gt; Parecer Médico&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção aparece na lista com o checkbox desabilitado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E ao passar o cursor aparece "Desabilitado para a faixa etária desse paciente"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o tooltip aparece apenas sobre essa opção</t>
         </is>
       </c>
     </row>
@@ -3341,6 +3621,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr"/>
@@ -3373,6 +3654,11 @@
       <c r="H117" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Manter a opção habilitada&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que &amp;lt;situação&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico acessa a tela de Solicitação de Pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção está habilitada e selecionável&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| situação                                              |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| a especialidade tem faixa etária e o paciente está dentro |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| a especialidade não tem faixa etária parametrizada    |</t>
         </is>
       </c>
     </row>
@@ -3395,6 +3681,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr"/>
@@ -3415,6 +3702,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr"/>
       <c r="H119" s="2" t="inlineStr"/>
+      <c r="I119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr"/>
@@ -3435,6 +3723,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr"/>
@@ -3467,6 +3756,11 @@
       <c r="H121" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Recalcular a idade ao abrir a tela&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o paciente completa a idade máxima da faixa hoje&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a tela de solicitação de pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a opção reflete a idade do dia da exibição</t>
         </is>
       </c>
     </row>
@@ -3489,6 +3783,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr"/>
+      <c r="I122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr"/>
@@ -3521,6 +3816,11 @@
       <c r="H123" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D4</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Bloqueio ao atingir o limite máximo de pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Exibir alerta com a relação de pareceres e apenas "Voltar"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a especialidade x filial tem limite máximo e comportamento "Sem justificativa (Trava Total)"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o paciente já possui pareceres em quantidade igual ao limite no período&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar um novo teleparecer dessa especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema exibe alerta informando que o limite foi atingido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E lista os pareceres do período com data, hora e responsável pela resposta&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E informa o tempo faltante para nova solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E disponibiliza apenas a opção "Voltar"</t>
         </is>
       </c>
     </row>
@@ -3543,6 +3843,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr"/>
+      <c r="I124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr"/>
@@ -3575,6 +3876,11 @@
       <c r="H125" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Comparar respondidos com o limite&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite máximo é &amp;lt;limite&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o paciente possui &amp;lt;respondidos&amp;gt; pareceres respondidos no período&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita novo teleparecer da especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a solicitação é &amp;lt;resultado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| limite | respondidos | resultado  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 2           | permitida  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 3           | bloqueada  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3      | 4           | bloqueada  |</t>
         </is>
       </c>
     </row>
@@ -3597,6 +3903,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr"/>
       <c r="H126" s="2" t="inlineStr"/>
+      <c r="I126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr"/>
@@ -3617,6 +3924,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr"/>
       <c r="H127" s="2" t="inlineStr"/>
+      <c r="I127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr"/>
@@ -3637,6 +3945,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr"/>
       <c r="H128" s="2" t="inlineStr"/>
+      <c r="I128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr"/>
@@ -3657,6 +3966,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr"/>
       <c r="H129" s="2" t="inlineStr"/>
+      <c r="I129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr"/>
@@ -3689,6 +3999,11 @@
       <c r="H130" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Voltar do alerta de Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado o alerta de Trava Total exibido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico clica em "Voltar"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então retorna à tela de solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E nenhuma solicitação é criada</t>
         </is>
       </c>
     </row>
@@ -3711,6 +4026,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr"/>
       <c r="H131" s="2" t="inlineStr"/>
+      <c r="I131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr"/>
@@ -3743,6 +4059,11 @@
       <c r="H132" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Solicitação com justificativa clínica ao atingir o limite&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Registrar a justificativa e criar o parecer&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite foi atingido e o comportamento é "Com justificativa"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o alerta exibe a lista de pareceres anteriores com data, hora e profissional&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico preenche a justificativa clínica e clica em "Prosseguir com a solicitação"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema cria o parecer normalmente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a justificativa fica vinculada de forma permanente à solicitação&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E está disponível no histórico/auditoria do paciente</t>
         </is>
       </c>
     </row>
@@ -3765,6 +4086,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr"/>
       <c r="H133" s="2" t="inlineStr"/>
+      <c r="I133" s="2" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr"/>
@@ -3797,6 +4119,11 @@
       <c r="H134" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Manter "Prosseguir com a solicitação" desabilitado&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado o alerta de limite atingido com justificativa&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o campo de justificativa contém "&amp;lt;conteúdo&amp;gt;"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o botão "Prosseguir com a solicitação" está &amp;lt;estado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| conteúdo       | estado       |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| (vazio)        | desabilitado |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| apenas espaços | desabilitado |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| texto válido   | habilitado   |</t>
         </is>
       </c>
     </row>
@@ -3819,6 +4146,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr"/>
       <c r="H135" s="2" t="inlineStr"/>
+      <c r="I135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr"/>
@@ -3839,6 +4167,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="2" t="inlineStr"/>
+      <c r="I136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr"/>
@@ -3859,6 +4188,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr"/>
       <c r="H137" s="2" t="inlineStr"/>
+      <c r="I137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr"/>
@@ -3879,6 +4209,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr"/>
       <c r="H138" s="2" t="inlineStr"/>
+      <c r="I138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr"/>
@@ -3911,6 +4242,11 @@
       <c r="H139" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Validar o tamanho da justificativa&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado o alerta de limite atingido com justificativa&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico informa &amp;lt;qtd&amp;gt; caracteres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o sistema &amp;lt;resultado&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o contador exibe &amp;lt;contador&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| qtd  | resultado                 | contador  |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 3999 | aceita                    | 3999/4000 |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 4000 | aceita                    | 4000/4000 |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| 4001 | impede a digitação/colagem além de 4000 | 4000/4000 |</t>
         </is>
       </c>
     </row>
@@ -3933,6 +4269,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr"/>
       <c r="H140" s="2" t="inlineStr"/>
+      <c r="I140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr"/>
@@ -3953,6 +4290,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr"/>
       <c r="H141" s="2" t="inlineStr"/>
+      <c r="I141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr"/>
@@ -3973,6 +4311,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr"/>
       <c r="H142" s="2" t="inlineStr"/>
+      <c r="I142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr"/>
@@ -3993,6 +4332,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr"/>
       <c r="H143" s="2" t="inlineStr"/>
+      <c r="I143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr"/>
@@ -4025,6 +4365,11 @@
       <c r="H144" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Desistir de prosseguir&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado o alerta de limite atingido com justificativa&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico clica em "Voltar"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então retorna à tela de solicitação de pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E não registra nova solicitação nem justificativa</t>
         </is>
       </c>
     </row>
@@ -4047,6 +4392,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr"/>
       <c r="H145" s="2" t="inlineStr"/>
+      <c r="I145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr"/>
@@ -4079,6 +4425,11 @@
       <c r="H146" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Não exibir a exceção quando o comportamento é Trava Total&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que o limite foi atingido e o comportamento é "Sem justificativa (Trava Total)"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico tenta solicitar&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o campo de justificativa e o botão "Prosseguir com a solicitação" não são exibidos</t>
         </is>
       </c>
     </row>
@@ -4101,6 +4452,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr"/>
       <c r="H147" s="2" t="inlineStr"/>
+      <c r="I147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr"/>
@@ -4133,6 +4485,11 @@
       <c r="H148" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidade: Lembrete de parecer recente&lt;br&gt;&amp;nbsp;&amp;nbsp;Cenário: Exigir o ciente para solicitar mesmo assim&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que existe parecer da especialidade dentro da janela do lembrete&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que o limite máximo de frequência ainda não foi atingido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico seleciona a especialidade e tenta solicitar&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então é exibido alerta com a data do parecer anterior&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a lista dos demais pareceres da janela com data, hora e profissional&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o checkbox "Estou ciente dos pareceres anteriores e reconheço a necessidade clínica de uma nova solicitação para este paciente."&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E o botão "Solicitar mesmo assim" está desabilitado até marcar o checkbox&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico marca o checkbox e clica em "Solicitar mesmo assim"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a solicitação prossegue</t>
         </is>
       </c>
     </row>
@@ -4155,6 +4512,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr"/>
       <c r="H149" s="2" t="inlineStr"/>
+      <c r="I149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr"/>
@@ -4175,6 +4533,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
+      <c r="I150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr"/>
@@ -4195,6 +4554,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr"/>
       <c r="H151" s="2" t="inlineStr"/>
+      <c r="I151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr"/>
@@ -4227,6 +4587,11 @@
       <c r="H152" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Esquema do Cenário: Não exibir o lembrete&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que &amp;lt;situação&amp;gt;&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita a especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o alerta de lembrete não é exibido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a solicitação segue normalmente&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Exemplos:&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| situação                                                                 |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| não existe parecer da especialidade dentro da janela do lembrete          |&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;| a especialidade x filial não possui janela do lembrete parametrizada      |</t>
         </is>
       </c>
     </row>
@@ -4249,6 +4614,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr"/>
       <c r="H153" s="2" t="inlineStr"/>
+      <c r="I153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr"/>
@@ -4269,6 +4635,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr"/>
       <c r="H154" s="2" t="inlineStr"/>
+      <c r="I154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr"/>
@@ -4289,6 +4656,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr"/>
       <c r="H155" s="2" t="inlineStr"/>
+      <c r="I155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr"/>
@@ -4321,6 +4689,11 @@
       <c r="H156" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695; Pendente-refinamento; D8</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Janela do lembrete diferente do intervalo do limite&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado que a janela do lembrete é de 12 horas e o intervalo do limite é de 48 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E que existe parecer há 20 horas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita a especialidade&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o lembrete não é exibido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;E a contagem do limite considera as 48 horas</t>
         </is>
       </c>
     </row>
@@ -4343,6 +4716,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr"/>
       <c r="H157" s="2" t="inlineStr"/>
+      <c r="I157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr"/>
@@ -4375,6 +4749,11 @@
       <c r="H158" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Voltar sem solicitar&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado o alerta de lembrete exibido&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico clica em "Voltar"&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então retorna à tela de solicitação sem criar parecer</t>
         </is>
       </c>
     </row>
@@ -4397,6 +4776,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr"/>
       <c r="H159" s="2" t="inlineStr"/>
+      <c r="I159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr"/>
@@ -4429,6 +4809,11 @@
       <c r="H160" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Manter o fluxo de solicitação em especialidades não parametrizadas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado uma especialidade sem nenhuma parametrização nova&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico solicita o parecer&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então o fluxo atual segue inalterado</t>
         </is>
       </c>
     </row>
@@ -4451,6 +4836,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr"/>
       <c r="H161" s="2" t="inlineStr"/>
+      <c r="I161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr"/>
@@ -4483,6 +4869,11 @@
       <c r="H162" s="2" t="inlineStr">
         <is>
           <t>Trava-Teleparecer; EF-1276695</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>Cenário: Abrir a lista com todas as regras ativas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Dado uma filial com muitas especialidades parametrizadas&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Quando o médico abre a Solicitação de Pareceres&lt;br&gt;&amp;nbsp;&amp;nbsp;&amp;nbsp;&amp;nbsp;Então a lista carrega em tempo aceitável, com cada opção validada</t>
         </is>
       </c>
     </row>
@@ -4505,6 +4896,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr"/>
       <c r="H163" s="2" t="inlineStr"/>
+      <c r="I163" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>